<commit_message>
auto: snapshot 2026-09-13 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -80,6 +80,7 @@
     <sheet name="2026-09-10" sheetId="72" state="visible" r:id="rId72"/>
     <sheet name="2026-09-11" sheetId="73" state="visible" r:id="rId73"/>
     <sheet name="2026-09-12" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="2026-09-13" sheetId="75" state="visible" r:id="rId75"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -52976,6 +52977,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-13 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>11103</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>+2951</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>+2902</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>+3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-13 05:05:58
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -53007,11 +53007,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Timestamp: 2026-09-13 13:00:10</t>
+          <t>Timestamp: 2026-09-13 13:05:56</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>11103</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
auto: snapshot 2026-09-14 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -81,6 +81,7 @@
     <sheet name="2026-09-11" sheetId="73" state="visible" r:id="rId73"/>
     <sheet name="2026-09-12" sheetId="74" state="visible" r:id="rId74"/>
     <sheet name="2026-09-13" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="2026-09-14" sheetId="76" state="visible" r:id="rId76"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -53865,6 +53866,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-14 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-15 05:00:17
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -82,6 +82,7 @@
     <sheet name="2026-09-12" sheetId="74" state="visible" r:id="rId74"/>
     <sheet name="2026-09-13" sheetId="75" state="visible" r:id="rId75"/>
     <sheet name="2026-09-14" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="2026-09-15" sheetId="77" state="visible" r:id="rId77"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -54754,6 +54755,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet77.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-15 13:00:15</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-16 05:00:12
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -83,6 +83,7 @@
     <sheet name="2026-09-13" sheetId="75" state="visible" r:id="rId75"/>
     <sheet name="2026-09-14" sheetId="76" state="visible" r:id="rId76"/>
     <sheet name="2026-09-15" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="2026-09-16" sheetId="78" state="visible" r:id="rId78"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -55643,6 +55644,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet78.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-16 13:00:10</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-17 05:00:11
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -84,6 +84,7 @@
     <sheet name="2026-09-14" sheetId="76" state="visible" r:id="rId76"/>
     <sheet name="2026-09-15" sheetId="77" state="visible" r:id="rId77"/>
     <sheet name="2026-09-16" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="2026-09-17" sheetId="79" state="visible" r:id="rId79"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -56532,6 +56533,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet79.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-17 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6451</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-19 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -86,6 +86,7 @@
     <sheet name="2026-09-16" sheetId="78" state="visible" r:id="rId78"/>
     <sheet name="2026-09-17" sheetId="79" state="visible" r:id="rId79"/>
     <sheet name="2026-09-18" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="2026-09-19" sheetId="81" state="visible" r:id="rId81"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -59167,6 +59168,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet81.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-19 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6751</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+300</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
auto: snapshot 2026-09-20 05:00:10
</commit_message>
<xml_diff>
--- a/clan_2527.xlsx
+++ b/clan_2527.xlsx
@@ -87,6 +87,7 @@
     <sheet name="2026-09-17" sheetId="79" state="visible" r:id="rId79"/>
     <sheet name="2026-09-18" sheetId="80" state="visible" r:id="rId80"/>
     <sheet name="2026-09-19" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="2026-09-20" sheetId="82" state="visible" r:id="rId82"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -60056,6 +60057,894 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet82.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D58"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Clan: Clairvoyant (2527) | S64</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Day Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Timestamp: 2026-09-20 13:00:09</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Total Reps</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Daily Reps (+1d)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nidzaa</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>24115</v>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Ninaa</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>23988</v>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>oy</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>24095</v>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>ReiKyuu X</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>6952</v>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>+201</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Mahsuri</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1031</v>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Parameswara</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Hang Tuah</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>942</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Mahawangsa</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Tun Teja</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>903</v>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Elavoth</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>899</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Dracoth</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>883</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Summoth</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>873</v>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Maximoth</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>865</v>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Shadow</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Assassin</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Zenith</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Astraphel</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Noir</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Lotus</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>AnbuMaster</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1229</v>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Zerofire</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>238</v>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Dominator</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>904</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Poseidon</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>iZengotsou</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1184</v>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>LotusEcstatic</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1019</v>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Aqua Lotus</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1144</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Legion Ape</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>987</v>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Heracoth</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>852</v>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HF Â·  SinBaD</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1308</v>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Tempest</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1406</v>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>SuPeR_TrIpLe</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1416</v>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Mercida</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Digipic</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>1264</v>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>$oloZ</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1272</v>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Aeternum</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1202</v>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>ID | [Let]hany</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>637</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Gawr[Gura]</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>1448</v>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>A Z</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>1278</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>A[n]Ton</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>934</v>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Bharat.</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>1442</v>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>A-S-H</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>1033</v>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Am_Ir</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Sovereign</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>851</v>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Ascendant</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>829</v>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>Harbinger</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>805</v>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Vanquisher</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>771</v>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>727</v>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Hera</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>780</v>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Athena</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>750</v>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>Artemis</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>729</v>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Aphrodite</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Hestia</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>700</v>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>K.aminari</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>A.stro</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>ras[E]n</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>